<commit_message>
Switch the applier from Muse to Grok Bot and rewrite the README
Add the grok-applier skill and a Grok Bot setup guide, replacing the
Muse guide. Update the setup prompt, checklist, kit and workbook to
match. Make the README accurate about what runs automatically and
what the agents' rules guarantee, and drop the banner, diagram and
badges.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workbook/agent-workbook.xlsx
+++ b/workbook/agent-workbook.xlsx
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>The shared workspace every agent (Claude, Muse, any other applier) and the human work through. Agents read this tab first and follow it exactly.</t>
+          <t>The shared workspace every agent (Claude, Grok Bot, any other applier) and the human work through. Agents read this tab first and follow it exactly.</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>[e.g. claude = role finder + inbox listener; muse = applier]. Each agent writes its own name in Owner fields.</t>
+          <t>[e.g. claude = role finder + inbox listener; grok = applier]. Each agent writes its own name in Owner fields.</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Claim before touching any application form. To claim: set State = claimed, Owner = your agent name, Claimed at = now (UTC), then read the row back. If the row changed under you or someone else's name is there, release nothing and pick a different role. Editing a row someone else owns is never allowed.</t>
+          <t>Claim before touching any application form. To claim: set State = claimed, Owner = your agent name, Claimed at = now (UTC), then read the row back. If the row changed under you or someone else's name is there, release nothing and pick a different role. Editing a row someone else owns is never allowed. To release a role you own and haven't applied to: set State = queued and clear Owner and Claimed at, then log it. A queued row never has an Owner.</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>muse</t>
+          <t>grok</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>muse</t>
+          <t>grok</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>muse</t>
+          <t>grok</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>muse</t>
+          <t>grok</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>muse</t>
+          <t>grok</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>muse</t>
+          <t>grok</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>